<commit_message>
Update example test file AddingDataTableAsWorksheet.xlsx
Update reference test file for example AddingDataTableAsWorksheet.xlsx.
After the style infrastructure switch, the styles part is saved differently.

The new file doesn't have dxf that was created due to original behavior
that checks consistent style of all data rows. That was from old behavior
that is likely going to be removed (there is a todo in TablePartWriter).
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Misc/AddingDataTableAsWorksheet.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Misc/AddingDataTableAsWorksheet.xlsx
@@ -61,73 +61,53 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="1">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="2">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="2">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-  <x:dxfs count="1">
-    <x:dxf>
-      <x:numFmt numFmtId="14" formatCode="M/d/yyyy"/>
-    </x:dxf>
-  </x:dxfs>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -137,7 +117,7 @@
     <x:tableColumn id="1" name="Dosage"/>
     <x:tableColumn id="2" name="Drug"/>
     <x:tableColumn id="3" name="Patient"/>
-    <x:tableColumn id="4" name="Date" dataDxfId="0"/>
+    <x:tableColumn id="4" name="Date"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>

</xml_diff>